<commit_message>
Finalize notebooks, evaluation results, and error analysis
</commit_message>
<xml_diff>
--- a/results/error_analysis/misclassified_clean_annotate.xlsx
+++ b/results/error_analysis/misclassified_clean_annotate.xlsx
@@ -434,7 +434,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>predicted_probability</t>
+          <t>pred_prob</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -451,7 +451,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Yes, these headphones are designed well to keep the sweat out of your ears. I bought them to replace the yellow "Sports" in-ear phones that came with my old cassete/radio Walkman. With those I had to take them out every once in a while and wipe the sweat off. With these new ones, it's not a problem.  However... I'm disappointed with the sound quality. I think it's because the in-ear part is bigger than it used to be - it doesn't go into my ear as far as the older model did. And they hurt! After about half an hour they make my ears hurt so bad that I have to give up on them. The fold-up feature and sweat guard design is not enough to justify the discomfort and lack of sound quality. I would not buy these again and recommend that other shoppers look elsewhere.  I'm training for a half-marathon and am still trying to find the perfect pair of traning earphones!!</t>
+          <t>This was the third Logitech trackball I've owned.  Like the other reviewers, I am a lefty, however I am a righthanded mouser.  My previous one was the TrackMan Vista which fit my hand like a glove and the buttons were in the exact right place when I put my hand on it in a natural position.  I'd still be using it if the sensors hadn't worn out from age, use and dust.  This trackman was stiff to use and I had to keep shifting my hand to hit the buttons. It did not install easily and would not connect using the ps2 adaptor so I was forced to use the usb connector and for some reason that caused issues with activesync so that every time I put my pda in it's docking station - the cursor would freeze.  Trying to get some real support from Logitech was a joke.  I finally had enough after 4 days of this and went to a big box electronic store and ended up buying a Microsoft Optical Trackman Explorer.  I am much happier as it is closer to the Vista than anything Logitech makes now.  It loaded easier, is more responsive and doesn't cause the issues the Trackman Wheel did.  The Logitech will be in my next garage sale if anyone is interested.</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -461,7 +461,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9990301962020787</v>
+        <v>0.3640685943581768</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -469,7 +469,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>I have a couple of these yellow anti-static wrist bands and I was teaching my kid about static electricity while doing a build.  I put the ohm meter to it and...no connectivity.  Unbelievable.  I've used this pair for years on my bench and I thought I must have worn out a connection in the head.  Nope.  When I grabbed my seldom used portable bag and tested the pair in there, same issue.  I tried wiggling them to see if maybe there was just a short in the connection and...Nope.  Simply unbelievable.  It's a good thing I always try to keep a hand on the chassis, exactly the way I was taught before these things were invented.  Needless to say I've ordered replacements and that Belkin has left a really sour taste in my mouth.</t>
+          <t>It just makes everything darker,  does not seem to retain color,  maybe for really special needs</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -479,7 +479,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7309620526475846</v>
+        <v>0.4038943163999319</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -487,17 +487,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The build quality is terrible! The glass is loose inside the ring and has lots of imperfections. Completely useless.</t>
+          <t>I could not figure out why my HD would go out, at times. Cable came out 2wice. Nope, nothing wrong. Must be your TV. I didn't think it was that. When I started rebooting, unplugging, etc., I noticed my plugs were a little loose on my power surge protector. So I figured that was it. I bought this and voila!! That was it. My plugs fit so snug in this thing. I LOVE Belkin anyway. What I had was Phillips. Stay AWAY from Phillips products. Any of them. I bought an electric toothbrush from them and I didn't have a receipt and Phillips wouldn't help me out at all. The battery was shot (before I ever used it!) and they wouldn't replace. They are a lousy company. They've been around forever and are NOT customer friendly and make LOUSY PRODUCTS. Stick with Belkin. All my wires are in the outlet now instead of on the floor. More space and tidier.</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9479091332982569</v>
+        <v>0.0414170096242962</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -505,17 +505,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>I have been in the entertainment industry for thirty five plus years .. Watching to pros around me use these headphones must have stuck in my head .. I just started a new business, needed headphones and the MDRV600s became the obvious choice .. They are comfortable to wear - Have a long cable and seem to reproduce a fine spectrum of natural sound .. I love these things .. I just wonder why I waited this long .. I should have had these to listen to my music a long while ago - There great!</t>
+          <t>I've heard lots of good things about Tiffen, but this may be imitation. The lens I received appeared used. It was scratched all along the edges, where the tint reaches the sides of the lens frame. A tiny bit of this is natural, but this is quite a lot; it will hurt my photo quality at the high resolution I take them with. It was also cloudy and I could never get it very clean, even with a lens cleaner applied several times.</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.004356390200329499</v>
+        <v>0.239110501848903</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -523,7 +523,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>It doesn't make a tight connection.  Any slight movement causes it to click, pop, and make disconnection noises.</t>
+          <t>the wipes are relly dry . i wish they were moistened a bit more</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -533,7 +533,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8757077702110782</v>
+        <v>0.6590257518396335</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -541,17 +541,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Once I downgraded the firmware (came with 1.40.1 and download was 1.39.2) worked GREAT!!  Good reception throughout my 1000 sq ft condo.  Very cool to sit on my couch, laptop in hand with no cords/cables and be able to surf the net.</t>
+          <t>The polarizing power is so weak that under many circumstances it is difficult to know whether it is rotated to the right position.</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.08014950045801374</v>
+        <v>0.473841918757167</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -559,17 +559,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Broke within the a week. Cheaply made. Was hoping this would be a quality splitter. I'd look elsewhere for an 3.5mm audio splitter.</t>
+          <t>I loved my SRIII.  Solid sound quality, excellent AM receptivity (but only average FM receptivity).  But it wasn't very hardy.  I took it camping once, and it was never the same after that.  It took several minutes to "warm up" after you turned it on, and then the sound was distorted for several minutes after that.  And scratchy sounds came out of the speaker when you adjusted the volume.  I figure the radio didn't like the humidity of the day and the dew of the morning.</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4038943163999319</v>
+        <v>0.1124091359144351</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -577,17 +577,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Inexpensive switch makes my life easier. Also cheap enough to use as drink coasters.</t>
+          <t>Mine came with little scratches and looks used... i think i will better stay using hoya... this tiffen was not nice.. more over it has a little warm tint, nothing so noticeable in pics, but it has some tint, it isn't neutral color</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0414170096242962</v>
+        <v>0.2445804528468916</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -595,7 +595,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ordered it back in Dec '11 and still waiting this filter to arrive. I'm with US Army and stationed overseas, so I typically expect shipping to be delayed.. but in this case after 2 months of waiting I would have to say this is either never sent by the seller or some how got lost in the mail. Not sure what I can do in this case.. so if Amazon customer service can able to help track this, I'd greatly appreciate it! Tks, Bon</t>
+          <t>I was expecting too much for the inexpensive price. However, the lens caps are so poorly formed that they fall off the small side lens by mere gravity. A light breeze could blow them right off. It isn't really worth the trouble to send them back so I will figure out a way to make the lens caps to stay where they are supposed to and I will use some kind of lanyard to keep them attached to the binoculars whether they are covering the lenses or not. My father has a pair that has this feature that he purchased in the early 1960's. It would cost a few cents per pair to incorporate this simple yet useful feature. The optics are what is to be expected from a $30.00 pair of binoculars which is not so good, but good enough to satisfy my meager needs. Something I will take with me when I go hiking. I gave two stars because of the lens caps.</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -605,7 +605,7 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9849334281509829</v>
+        <v>0.6219923396441757</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -613,7 +613,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Does not have much mid range and it is not comfortable.</t>
+          <t>The Good:  I really like the functionality and ergonomics of this pointing device. My wrist and arm stay much more relaxed. It did take a few days to train my thumb to be sensitive enough to place the cursor exactly where I wanted it. The optical ball operates smoothly and seems insensitive to dirt/oil build up. There are the usual left and right mouse buttons along with a scroll wheel. The scroll wheel also operates a third button. If you need more buttons, this device may not be for you. The supplied driver software allows the buttons to be programmed and the cursor speed, acceleration, etc, to be adjusted -- standard mouse stuff. I run a 1600x1200 21" monitor so have the acceleration set to High (max) and speed set to medium or just above. This allows me to move the cursor from corner to corner in just over a single thumb flick. However, I do experience a bit of difficulty placing the cursor accurately in close work. (See additional comments on this below.)  The Bad:  I bought my first Logitech Cordless TrackMan Wheel last fall to go with a new desk-side PC. Several months later it failed and rather than deal with the hassles of the Logitech warranty process over a $35 or so part, I just wrote it off as an early-life failure and bought another one. It failed yesterday (5/7/10). Now two failures in less than a year on a device which is claimed to have a 5 year warranty seems a bit much. Both of these were bought at a local electronics store, not Amazon -- arguably my bad. I read another review on this device where the reviewer had also experienced two failures.  So I bought yet another TrackMan Wheel yesterday, but this time the corded version since my desk set-up doesn't really require cordless. My initial observation is that with the same settings as indicated above, it is noticeably easier to accurately place the cursor -- cursor movement is smoother. Also, no battery is required though battery life in the cordless version is not an issue. BTW, I find the Minesweeper and Free Cell games to be readily available tools for checking out pointing devices.  Recommendations:  I would like to give this device a 5 star rating and recommend it highly. However, given the high failure rate I have experienced, I cannot do so.</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -623,7 +623,7 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5506860605293321</v>
+        <v>0.4113855846496335</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -631,17 +631,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>My favorite lens its picture quality and compact size. In a DX camera you will be looking into a 75mm 1.8; You couldn't find a better portrait lens!!  Build quality is below average. The lens barrel feels plasticky and flimsy - the "Made in China" tag seems to explain all. Fortunately the picture quality seems pretty good.  At this price - this is a steal!!</t>
+          <t>If you are going to be unplugging and plugging. Dont get them. They break easy and loses connection. I just purchased the MediaBridge ones. It is more money but look at the review I left it. Dont want to badger this one. If its a one time gig, I would say this one is reliable.</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02113826687518424</v>
+        <v>0.2054546281378656</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -649,17 +649,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>I am very pleased that I could get quality headphones at such a reasonable price. They will be a welcome addition to my listening pleasure.</t>
+          <t>I bought these manily becasue they were cheap and i at the time have gotten so sick of ear buds. They worked ok for two weeks then all of a sudden there was no sound coming from the right side. Another thing that is a big negative is that they are so dam big and ugly. If you go out in public with these you look like a out of date dork. Sony has gotten down hill lately with these breaking and a portable cd player i had that broke down in a couple of months. I remeber when sony used to make the best electronics. They were the ones that invented the walkman. There walkmans from the 90s and before were so great i still have one that i got 10 years ago.</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>0.03333565882335209</v>
+        <v>0.4189094218447188</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -667,17 +667,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>This is a cheap UV filter and if you are only using the 50mm f/1.8 lens to shoot indoor portraits, don't bother with this.</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>0.002258368440828227</v>
+        <v>0.3275012260787609</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -685,7 +685,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Great product</t>
+          <t>this is not a self pealing tape.</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -695,7 +695,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01338870355392324</v>
+        <v>0.05308965227166198</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -703,17 +703,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Item delivered on time, was as described.</t>
+          <t>They don't fit in my ear. They keep falling right out and i usually wear earplugs which never fall out.</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>0.08342976634718652</v>
+        <v>0.3122492199678298</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -721,7 +721,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>You get what you pay for. Not much else to say. They do the job nicely.</t>
+          <t>This review is aimed at those with eyeglasses and whose ears get pinched between the eyeglass arms and the earphones. I do not like to block up my ears with ear plugs all day for health concerns. I have bought and used these:  Sony MDR-CD230  Sony MDR-V6  Sony MDR-XD200  My ears are not real fussy on quality, nearly all headphones give my ears a problem by pressing them against my eyeglass arms and this hurts, usually after 10-20 minutes of listening. My hatsize if about 7.25,  my ears are pretty normal in size, I am middle aged. All three of these headphones I own are the best I have tried on or read reviews by eyeglass wearers over past 2 years. Headphones have a left and right side - the cord typically is attached to the left side, and the ear spaces, or cups, are oriented accordingly, to that the back of the ear lobe has more space to sit in than the front of the ear lobe. The sideways pressure (how hard they clamp onto your head) also is a secondary factor in whether my ears hurt. I wear wireframe glasses, and my use for headphones is background music while I program.  $30 The CD230 is no longer available, that I could find (Fall 2006), and I've used them for 5 years. They hurt my ears after 3-4 hours of continual use, but are good before that. They have cloth covered ear cushions, and relatively deep ear lobe spaces. This feature in all earphone seems to be the primary feature that determines whether my ears hurt or not. If you can find these, and like cloth covered headphones, you won't be unhappy. The sideways pressure is light for me.  $64 The V6 stands out for 2 things - richness and accuracy of the sound and blocking out outside office noises. Listening to classical music, not real loud, a co-worker can speak to my face and his voice is muffled pretty well. (Women's voices too). Overheard conversations are not overheard.  I have used these occaisionally for a couple months and my ears/head get sore after 1-2 hours. The sideways pressure is noticeably more than the other two, but not excessive. They are well cushioned, with soft fake thin leather-like vinyl which I did not find causes sweating at all. But there is not a large space for the ear lobes to sit, and this is what causes pressure after a while to build up uncomfortably I am sure. If I did not have my eyeglasses on, then these are very comfortable.  $26 The XD200 is a little lighter than the V6, it does not block out outside noises as well, which can be a benefit in the office because I can hear co-workers calling my name. The sideways pressure is light, the cushion is the same thickneess as the V6 but the ear space is much deeper for the earlobe, so for this reason it is the most comfortable of all headphones I've owned or tried. The cushions are covered in the thin leather-like vinyl like the V6 - this stuff feels like a paper much more than a plastic, it feels dry, not clammy. To my unprofessional ears the sound is great. If you wear eyeglasses, don't want to use ear plugs for hours at a stretch, then I think you will be happiest with the Sony MDR-XD200 headphones.</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -731,7 +731,7 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0.008388295755410885</v>
+        <v>0.1436007588196319</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -739,7 +739,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>This doesn't work with analog joysticks on Windows 10.  Not impressed.</t>
+          <t>Set up the speakers but no sound from the right speaker.  I then called Klipsch and they had me connect my earphones to the right speaker and sound came through both earphones...the tech support individual indicated the amplifier is blown.  He stated the speakers probably got banged around in shipping??????</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -749,7 +749,7 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>0.9970295051179635</v>
+        <v>0.3118521650461081</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -757,17 +757,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GOOD CABLE WORKS AS IT IS SUPPOSED TO HAS A GOOD CONNECTION (GRIP) ON IT AS WELL.</t>
+          <t>These deliver a  lot of power, but it's all in the lowever frequencies. The mids are the most important part of the audio spectrum, and these just don't cut it. The high frequencies add snap, and these do well enough but without going through a graphic equalizer, you lose. So for music, you need a player with a graphic equalizer, and you must attenuate the low frequencies, boost the mids, and boost the last two high sliders even more. You also need to raise the bass volume from 0 to about 5%, and no more! More than this really distorts the out[put of all frequencies.  Bottom line, these are bass rich.... far too bass rich.  I have a lot of music. It comes in all flavors from Classical to Rock. I even have music from around the world. These speakers do okay but you MUST have a graphic equalizer. Both Winamp and iTunes have one built in, but YouTube does not, and YouTubes that I know are in good condition sound pretty awful. You wind up with a mix of distortion and frequency bleed. There is a fix, however. There's a free wareapp that allows you to set all system sounds with a 12 slider graphic equalizer that runs behind evrything. It also has a preamp built in. So what you can do is run this, and set it to the settings on your Winamp player, then have this preamp boot upon Windows boot up, then flatten your iTunes and Winamp equalizer. The result is the same.  Overall though, these are far too bass rich. And the volume knobs cause distortion at BEFORE the 50% mark, so these don't go all that loud thanks to the distorion that's inherently built in. But most people sit at the computers with their speakers nearby, so you don't need a lot of volume most of the time, but when you do, you get that volume and a hella lotta distortion in all frequencies.  Don't be fooled. If you have a chance to preview these, make sure you have music the has a real piano, violins, accoustic guitars, and just plain real instruments. You can get the sound balanced, but it's a rather lengthy trial and error to get your equalizer set correctly. But once set, these deliver aqequate sound, but not as loud as the volume controls allow, because even if that equalizer is left alone, you can only get about 50% of the volume out of these before distortion becomes VERY apparent.</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>0.003150258769961319</v>
+        <v>0.6239833945092419</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -775,17 +775,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>I am watching Dish tv at the sound level I need without bothering my wife.</t>
+          <t>At first I thought this was a good product. It felt sturdy and genuinely well made. After I started filling it up though I noticed that the movies that had been on the bottom row of the case for a while started getting scuff mark above the title. I looked at about 15 dvds on the bottom row and they all had the scuff marks. I didn't realize this little plastic edge from part of the holder on the top row sticks down and is pretty sharp. Well it seems I found this out the hard way because now im not sure if i can watch the end of any of my movies. This is really irritating and i feel like they just cheaped out on the production line and didn't make the sleeves big enough.  By this if product if you feel like doing precision surgery on every page to cut the little flap of destruction off.</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1162509504404669</v>
+        <v>0.2347452559980191</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -793,17 +793,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Great headphones. We have an older set of this same pair of headphones so we felt confident ordering this brand. We were happy to see they are still well made.</t>
+          <t>This product will work with windows 98 however much tweaking is needed and many hours on tech support. One thing I will say is this  adapter randomly decideds which XP computers it wants to work on. I have it configured corectly but why make a product that goes against windows thats made for windows? If you ask me you should have to configure it to work against windows not the other way around!</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>0.01000924585437514</v>
+        <v>0.2333775915680499</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -811,7 +811,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>You can barely hear anything that comes out of these speakers.  They were a waste of money and I regret it.</t>
+          <t>I wanted to like this lens because I always prefer lenses with a close focusing distance, and this is a rare macro 28mm (not a "true macro" but it focuses very close). Unfortunately I was never satisfied with the image quality of the photos. The lens is mush wide open, and it never gets really sharp across the board, even when stopped down. The bokeh has an ugly swirly quality that makes the background of close-ups unpleasant looking. It might be OK for landscape shots of mountains, etc. when used close to infinity and stopped way down, but then what's the point of having a fast "macro" lens if you can't use it at the wide apertures and minimum focus distance?  I used it on a full frame camera but it would make a good "normal" focal length lens on a crop sensor camera, if the optics were better. Instead I would opt for the Sigma 30mm f/1.4 lens which is actually usable wide open. Sigma has some great lenses but this isn't one of them. Unlike another reviewer, I found the build quality and autofocus performance to be just fine, but the optics to be sub-par; others have found the opposite.  If you are going to buy only one wide angle lens, make it the&amp;nbsp;&lt;a data-hook="product-link-linked" class="a-link-normal" href="/Zeiss-21mm-f-2-8-Distagon-T-ZE-Series-Lens-for-Canon-EOS-Digital-SLR-Cameras/dp/B002UBPWAK/ref=cm_cr_arp_d_rvw_txt?ie=UTF8"&gt;Zeiss 21mm f/2.8 Distagon T* ZE Series Lens for Canon EOS Digital SLR Cameras&lt;/a&gt;. Yes, it costs a small fortune, but it's worth every penny. Sell some other lenses if you have to; the Zeiss 21 can replace all of your wide angle lenses, it's so good--even if you need to crop them a bit to a 24 or 28mm field of view. There is something very special and even magical about the Zeiss 21 that has to be experienced; it makes you not want to use any other wide angle lens once you've tried it.</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -821,7 +821,7 @@
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>0.9377587570481019</v>
+        <v>0.5155909414233675</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -829,7 +829,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Doesn't have the muscle for cold 12guage I use for my electric snow blower. It just can't grip the cord. May be fine for std extension cords.</t>
+          <t>I typically want a case that will cary 1 or 2 sets of spare, AA Batteries, Plympus SmartMedia cards, camera and possibly my AC Olympus charge when I fly to various photo sites.  This case is simply too small for that.</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -839,7 +839,7 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>0.7621500485066353</v>
+        <v>0.7908785709303789</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -847,7 +847,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>This product does not have caller ID and makes a hissing sound that is irritating. I bought it from BuyAccessories, who were great with customer service and refunded my purchase. I will buy from them again. It's not their fault the product is mediocre.</t>
+          <t>Had difficulty understanding each other with these. When using the walkie talkies directly they were fine, but with these the sound was muddled and very difficult to understand at times. Probably discontinued for a reason.</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -857,7 +857,7 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9895989004338852</v>
+        <v>0.4164475738824524</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -865,7 +865,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>This cable really isn't that flat - it's about 2 to 2.5 mm (1/10th inch) thick, and 14mm (0.55 in) wide.  (The thickness dimension at the Monster site is wrong.)  Not really enough thinner than regular wire, and not space-efficient (see below).  It may be best for running along baseboards, etc.  It's a little too thick to run under most carpets, or to paint and have it actually disappear.  Monster doesn't like to tell you the gauge of cables, but these are 16 AWG.  Which is just fine for up to about 40 feet, maybe more.  Google speaker wire for some discussion on what size wire you need for a given distance from the receiver to the speaker.  The design could be improved, maybe that's why these are sharply discounted lots of places.  As noted, they aren't at all Superflat.  There's a chunk of plastic down the center that seems unnecessary - maybe it's there to provide a place to attach (nail, screw, staple), but it's just taking up space that could have been used to make the wire flatter instead.  If you're willing to pay a lot more (about $1/foot) you can get truly flat speaker wire.  But, since this cable is available for a fraction of list if you look around, it might suit your needs for a specific installation.  The color is an off-white, with a slightly yellowish tinge.  Sort of a cream color.  But - and here's another design flaw - one wire is marked on one side with a silver line, with "Superflat Mini" and a bunch of other text every foot.  It's much more than is needed to mark the polarity of the wire (to make sure you connect + to + and - to - on the speakers).  So it means that only the unmarked side of the wire is really usable - a 90 flat turn on a surface flips the text out onto the exposed side of the wire - unless you plan to paint this.  The SFLM GP50 package includes 4 red/black pairs of straight termination pins, crimp to attach.  They don't seem designed for this wider wire, though - they're really meant for standard round wire.  There are also 4 clamps (to hold the wire to the wall) and 2 "corner trim" pieces (for making a 90 turn by folding over the wire and putting it into the trim).  Not enough clamps for a whole run, if you use them, but might be handy.  File this under products that could be a lot better.</t>
+          <t>Not recommended since it damages your video equipment</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -875,7 +875,7 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0.9998171059519733</v>
+        <v>0.4650090656894488</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -883,7 +883,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Only works for a little while, then the dirty electric comes back....  Would recommend and APC UPS instead.</t>
+          <t>One of Nikon's worst lenses. Terrible distortion around the edges on wide open shots. Great macro lens though.</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -893,7 +893,7 @@
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0.9334687039202979</v>
+        <v>0.4368189269393776</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -901,17 +901,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Well I have to admit I was wrong about Cordless Keyboards. It's pretty convenient being able to sit back in your chair with the keyboard on your lap facing the TV...and still be able to write emails. The sensor is EXTREMLY sensitive, and the keyboard doesnt haev to be pointed in the direction of it at all to work fine. The mouse is heavy. It's got 2 batteries in it, and obviously has plenty of electrical hardware inside to make it wireless capable. Its shaped for your hand nicely, but if your going to be playing games (mainly first person shooters), this isn't a GREAT mouse. Its heavy, and a little slow. I liked my wired Logitech Optical mouse better for games. If your NOT playing games, you'll probably find the mouse to be a perfect fit for your needs, especially if your going from a "track ball" mouse, which in my opinion is the most annoying thing you could have on a computer. (You'll agree with me once you use an optical). Overall, for the sale price that amazon has it for, it's a pretty good deal. It looks VERY nice..black and silver color combo. The best looking keyboard/mouse combo I could find. It works well, but as usual I'm having trouble with the "I touch" function, which are the hot keys. They work sometimes, and other times they don't. I don't feel the need to use them anyway, so that isn't a concern. Overall another quality product from Logitech. This is one reliable company in the world of computer hardware. I've had nothing but good experiences with them, and this is another. I originally bought an internet keyboard, but opted for this set with my new 2.8ghz Dell 8200 system. (I'm a pretty hardcore gamer) Good luck and take care.</t>
+          <t>Dis one, she no good mon. Last mebe, what? 3 monts zall. I buy 3 but don buy no mo.</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1124091359144351</v>
+        <v>0.4706248896664804</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -919,17 +919,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>I'm transcribing interviews and this machine is excellent.  With the foot pedal back-track, I can listen to the speaker as often as I need to without lifting my hands off my keyboard.</t>
+          <t>I was laying down on my couch in my HT room and was awakened by a loud POP!  It was my sub blowing.  It had no signal going to it and nothing else was being used on that circuit at the time.  Luckily my Acoustic Research surge protector saved my DLP, Receiver, and Xbox 360.</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>0.006813319889971174</v>
+        <v>0.8320860969267001</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -937,17 +937,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>As I was finding myself getting ready for a long couple of weeks of temporary duty in Guatemala and in need of a good set of headphones for a portable DVD player to watch movies while sitting in a tent, I went to the trusted brand name of Sony.  The Sony MDR-V300 Traditional Collapsible DJ Style Headphones fulfilled this requirement in the usual wonderful manner that Sony products so often do. As I lay in the tent watching movies with these outstanding headphones on, the audio tracks on the DVD's were played wonderfully, enhancing the movie watching experience to perfection, giving a theater style performance..  While these headphones do not drown out ambient noises completely as they're not advertised to do so, they do keep a majority of the ambient noises to a minimum making the experience that much better. For price and quality, one can hardly do better than to make the decision to purchase these outstanding headphones and I highly recommend them to any and all who find themselves in need of a good pair of headphones.  I expect to get several years of good use out of these headphones and have high confidence in the quality and high standard of performance in this, another outstanding Sony product!  {ssintrepid}</t>
+          <t>The product itself is no problem. I ordered a few more than I need and called right away to stop the order and was told that I can't even change my order to fewer quantity.</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>0.005793047001393796</v>
+        <v>0.3155030594629393</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -955,7 +955,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>This hub doesn't work with my headset or ipod. It needs a power adapter, which I haven't been able to find. Utterly useless without it.</t>
+          <t>I just got this item and installed it as directed.  But the film is too dark and doesn't work well for a wide 27" screen.  I can only see directly in front of my eyes and the edges of my screen are dark.  Not what I was expecting so I will keep looking for something that allows me to view my entire screen!</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -965,7 +965,7 @@
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>0.9967627424654606</v>
+        <v>0.2339886303697156</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
@@ -973,7 +973,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>The sound is muddy and the foam portion is designed in such a way that it is nearly impossible to seat the earpieces firmly to block out external sounds. I don't really know which characteristic bothers me the most.</t>
+          <t>I am a very technical person (I teach Photoshop) and this product is either defective, or I should have paid attention to the mediocre evaluations. We still cannot get the CD player to work. You should be able to hit CD, then play, and it should work. Buy a Sony instead. We have one for my son, and it's great. My daughter still has no music in her room.</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -983,7 +983,7 @@
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>0.8539073600467615</v>
+        <v>0.3012335446663978</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>

</xml_diff>